<commit_message>
lab5: competitor prices (Arixcel, Operis) recalculated in workbooks, reports rebuilt
</commit_message>
<xml_diff>
--- a/ЛР5_Анализ_конкурентов/Excel/ЛР5_1_классификация_по_уровням_конкуренции_TableMind.xlsx
+++ b/ЛР5_Анализ_конкурентов/Excel/ЛР5_1_классификация_по_уровням_конкуренции_TableMind.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-3ab569\ЛР5_Анализ_конкурентов\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР5_Анализ_конкурентов\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632393F5-3EBF-446C-B2AF-1D0E6E0CC751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E50E750-030A-4A2F-8F3D-26CA70262AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="368" yWindow="368" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1940,7 +1940,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FB79-4CFD-A141-7823D7DEA1D6}"/>
+              <c16:uniqueId val="{00000000-3EDE-4D17-A256-425B09B6FCD0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2380,7 +2380,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B802-481B-9146-6F15F19CD684}"/>
+              <c16:uniqueId val="{00000000-2E45-48DC-939A-0782822E97C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
lab5: methodology norms met (32 pages, 25 Kano features), recalculated workbooks (79 checks), report and docs rebuilt
</commit_message>
<xml_diff>
--- a/ЛР5_Анализ_конкурентов/Excel/ЛР5_1_классификация_по_уровням_конкуренции_TableMind.xlsx
+++ b/ЛР5_Анализ_конкурентов/Excel/ЛР5_1_классификация_по_уровням_конкуренции_TableMind.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TableMind_EB\.claude\worktrees\handoff-continuation-57ce20\ЛР5_Анализ_конкурентов\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E50E750-030A-4A2F-8F3D-26CA70262AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD107421-9AA0-4D17-85AC-A2FE4CE5DFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="458" windowWidth="12022" windowHeight="10972" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Инструкция" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="589">
   <si>
     <t>Методика работы с Excel-шаблоном классификации компаний по уровням конкуренции</t>
   </si>
@@ -1614,6 +1614,174 @@
   </si>
   <si>
     <t>Присутствует в магазине надстроек</t>
+  </si>
+  <si>
+    <t>Безопасность</t>
+  </si>
+  <si>
+    <t>https://www.datasnipper.com/security</t>
+  </si>
+  <si>
+    <t>SOC 2 Type II, Azure, AES-256, TLS 1.2+, хранение до 24 часов, обучение на данных клиентов не ведется, GDPR и AI Act</t>
+  </si>
+  <si>
+    <t>Самый подробный профиль безопасности среди специализированных игроков</t>
+  </si>
+  <si>
+    <t>https://www.datasnipper.com/pricing</t>
+  </si>
+  <si>
+    <t>Start, Accelerate, Elevate без сумм; Book demo и Contact sales</t>
+  </si>
+  <si>
+    <t>Цена по запросу, вход через демо</t>
+  </si>
+  <si>
+    <t>Интеграции</t>
+  </si>
+  <si>
+    <t>https://knowledge.datasnipper.com/en/collections/1449483-integrations</t>
+  </si>
+  <si>
+    <t>SharePoint, OneDrive, Box, Dropbox, SAP Concur, QuickBooks, Suralink, Azure</t>
+  </si>
+  <si>
+    <t>Интеграции документов аудита, не проверки формул</t>
+  </si>
+  <si>
+    <t>Отзывы Capterra</t>
+  </si>
+  <si>
+    <t>https://www.capterra.com/p/10002513/DataSnipper/</t>
+  </si>
+  <si>
+    <t>4,7 из 5, 131 отзыв, пробной версии нет</t>
+  </si>
+  <si>
+    <t>Сильный репутационный профиль</t>
+  </si>
+  <si>
+    <t>https://datarails.com/pricing/</t>
+  </si>
+  <si>
+    <t>Professional, Premium, Expert без сумм; Request Quote, пробного периода нет</t>
+  </si>
+  <si>
+    <t>Цена по запросу, длинный цикл продажи</t>
+  </si>
+  <si>
+    <t>Центр доверия</t>
+  </si>
+  <si>
+    <t>https://trust.datarails.com/overview</t>
+  </si>
+  <si>
+    <t>SOC 2 Type II, SOC 1, политика информационной безопасности, тест на проникновение; отчеты по запросу</t>
+  </si>
+  <si>
+    <t>Самый полный профиль доверия</t>
+  </si>
+  <si>
+    <t>https://datarails.com/integrations/</t>
+  </si>
+  <si>
+    <t>более 200 интеграций в списке (ERP, CRM, хранилища); на главной заявлено более 600</t>
+  </si>
+  <si>
+    <t>Интеграции - барьер переключения</t>
+  </si>
+  <si>
+    <t>https://www.capterra.com/p/177451/DataRails/</t>
+  </si>
+  <si>
+    <t>4,7 из 5, 245 отзывов</t>
+  </si>
+  <si>
+    <t>Лицензирование</t>
+  </si>
+  <si>
+    <t>https://www.arixcel.com/explorer/download</t>
+  </si>
+  <si>
+    <t>2,75 GBP за пользователя в месяц, лицензия 12-36 месяцев, только Windows, пробный режим</t>
+  </si>
+  <si>
+    <t>Цена опубликована, лестницы тарифов нет</t>
+  </si>
+  <si>
+    <t>Цены OAK</t>
+  </si>
+  <si>
+    <t>https://www.operisanalysiskit.com/oak-price/</t>
+  </si>
+  <si>
+    <t>подписка 311,66 GBP в год, более 30 инструментов, Try OAK и Buy now</t>
+  </si>
+  <si>
+    <t>Единичная цена, продажа без консультанта</t>
+  </si>
+  <si>
+    <t>https://shortcut.ai/privacy</t>
+  </si>
+  <si>
+    <t>SOC 2 Type II, AES-256, TLS 1.3, нулевое хранение у провайдеров, SAML, ролевой доступ</t>
+  </si>
+  <si>
+    <t>Безопасность раскрыта в центре приватности</t>
+  </si>
+  <si>
+    <t>Цены и регистрация</t>
+  </si>
+  <si>
+    <t>https://numerous.ai/</t>
+  </si>
+  <si>
+    <t>7 дней бесплатно, оплата за год, 10 USD в месяц, лимит 500 тыс. символов</t>
+  </si>
+  <si>
+    <t>Путь от пробы к подписке без продавца</t>
+  </si>
+  <si>
+    <t>Подвал сайта</t>
+  </si>
+  <si>
+    <t>только политика конфиденциальности и условия, заявлений о безопасности нет</t>
+  </si>
+  <si>
+    <t>Безопасность не раскрыта</t>
+  </si>
+  <si>
+    <t>Отзывы Trustpilot</t>
+  </si>
+  <si>
+    <t>https://www.trustpilot.com/review/numerous.ai</t>
+  </si>
+  <si>
+    <t>2,5 из 5, 5 отзывов, жалобы на автосписание после пробного периода</t>
+  </si>
+  <si>
+    <t>Риск политики пробного периода</t>
+  </si>
+  <si>
+    <t>Пробный период</t>
+  </si>
+  <si>
+    <t>https://www.perfectxl.com/products/perfectxl-formula-inspector/free-trial-vdependents/</t>
+  </si>
+  <si>
+    <t>30 дней без карты и автопродления, Excel 2016 и новее</t>
+  </si>
+  <si>
+    <t>Бесплатный вход есть</t>
+  </si>
+  <si>
+    <t>Правовые страницы</t>
+  </si>
+  <si>
+    <t>https://www.perfectxl.com/legal/privacy-policy/</t>
+  </si>
+  <si>
+    <t>политика конфиденциальности, условия, cookie; страницы безопасности нет</t>
   </si>
   <si>
     <t>https://rows.com/pricing</t>
@@ -1940,7 +2108,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3EDE-4D17-A256-425B09B6FCD0}"/>
+              <c16:uniqueId val="{00000000-3FAE-47FB-9A98-626F18B215E2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2380,7 +2548,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2E45-48DC-939A-0782822E97C6}"/>
+              <c16:uniqueId val="{00000000-A78A-4BA9-AAC2-A138F10E0A63}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5962,25 +6130,25 @@
         <v>475</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="27">
+    <row r="20" spans="1:12" ht="40.5">
       <c r="A20" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B20" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A20,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v>Rows</v>
+        <v>DataSnipper</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>476</v>
+        <v>524</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="G20" s="2">
         <v>4</v>
@@ -5989,7 +6157,7 @@
         <v>46298</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="J20" s="2">
         <v>5</v>
@@ -6001,23 +6169,23 @@
     </row>
     <row r="21" spans="1:12" ht="27">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B21" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A21,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v>Formula Bot</v>
+        <v>DataSnipper</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>504</v>
+        <v>476</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="G21" s="2">
         <v>4</v>
@@ -6026,10 +6194,10 @@
         <v>46298</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J21" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
@@ -6038,312 +6206,632 @@
     </row>
     <row r="22" spans="1:12" ht="27">
       <c r="A22" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B22" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A22,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v>Microsoft 365 Copilot</v>
+        <v>DataSnipper</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>476</v>
+        <v>531</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="G22" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H22" s="5">
         <v>46298</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="J22" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K22" s="2"/>
       <c r="L22" s="2" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
-      <c r="A23" s="2"/>
+    <row r="23" spans="1:12" ht="27">
+      <c r="A23" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="B23" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A23,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
+        <v>DataSnipper</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="G23" s="2">
+        <v>4</v>
+      </c>
+      <c r="H23" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="J23" s="2">
+        <v>5</v>
+      </c>
       <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-    </row>
-    <row r="24" spans="1:12">
-      <c r="A24" s="2"/>
+      <c r="L23" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="27">
+      <c r="A24" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="B24" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A24,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+        <v>Datarails</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="G24" s="2">
+        <v>4</v>
+      </c>
+      <c r="H24" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="J24" s="2">
+        <v>5</v>
+      </c>
       <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" s="2"/>
+      <c r="L24" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="40.5">
+      <c r="A25" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="B25" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A25,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+        <v>Datarails</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G25" s="2">
+        <v>4</v>
+      </c>
+      <c r="H25" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="J25" s="2">
+        <v>5</v>
+      </c>
       <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="1:12">
-      <c r="A26" s="2"/>
+      <c r="L25" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="27">
+      <c r="A26" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="B26" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A26,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+        <v>Datarails</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G26" s="2">
+        <v>4</v>
+      </c>
+      <c r="H26" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="J26" s="2">
+        <v>4</v>
+      </c>
       <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="1:12">
-      <c r="A27" s="2"/>
+      <c r="L26" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="27">
+      <c r="A27" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="B27" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A27,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+        <v>Datarails</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="G27" s="2">
+        <v>4</v>
+      </c>
+      <c r="H27" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="J27" s="2">
+        <v>5</v>
+      </c>
       <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-    </row>
-    <row r="28" spans="1:12">
-      <c r="A28" s="2"/>
+      <c r="L27" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="27">
+      <c r="A28" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="B28" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A28,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+        <v>Arixcel</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G28" s="2">
+        <v>4</v>
+      </c>
+      <c r="H28" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="J28" s="2">
+        <v>5</v>
+      </c>
       <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-    </row>
-    <row r="29" spans="1:12">
-      <c r="A29" s="2"/>
+      <c r="L28" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="27">
+      <c r="A29" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="B29" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A29,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+        <v>Operis</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="G29" s="2">
+        <v>4</v>
+      </c>
+      <c r="H29" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="J29" s="2">
+        <v>5</v>
+      </c>
       <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="1:12">
-      <c r="A30" s="2"/>
+      <c r="L29" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="27">
+      <c r="A30" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="B30" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A30,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
+        <v>Shortcut</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G30" s="2">
+        <v>4</v>
+      </c>
+      <c r="H30" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="J30" s="2">
+        <v>5</v>
+      </c>
       <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-    </row>
-    <row r="31" spans="1:12">
-      <c r="A31" s="2"/>
+      <c r="L30" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="27">
+      <c r="A31" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="B31" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A31,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
+        <v>Numerous.ai</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="G31" s="2">
+        <v>4</v>
+      </c>
+      <c r="H31" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="J31" s="2">
+        <v>4</v>
+      </c>
       <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-    </row>
-    <row r="32" spans="1:12">
-      <c r="A32" s="2"/>
+      <c r="L31" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="27">
+      <c r="A32" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="B32" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A32,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+        <v>Numerous.ai</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G32" s="2">
+        <v>4</v>
+      </c>
+      <c r="H32" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="J32" s="2">
+        <v>4</v>
+      </c>
       <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-    </row>
-    <row r="33" spans="1:12">
-      <c r="A33" s="2"/>
+      <c r="L32" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="27">
+      <c r="A33" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="B33" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A33,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+        <v>Numerous.ai</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="G33" s="2">
+        <v>4</v>
+      </c>
+      <c r="H33" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="J33" s="2">
+        <v>5</v>
+      </c>
       <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-    </row>
-    <row r="34" spans="1:12">
-      <c r="A34" s="2"/>
+      <c r="L33" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="27">
+      <c r="A34" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="B34" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A34,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+        <v>PerfectXL</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G34" s="2">
+        <v>4</v>
+      </c>
+      <c r="H34" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="J34" s="2">
+        <v>5</v>
+      </c>
       <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-    </row>
-    <row r="35" spans="1:12">
-      <c r="A35" s="2"/>
+      <c r="L34" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="27">
+      <c r="A35" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="B35" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A35,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+        <v>PerfectXL</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G35" s="2">
+        <v>4</v>
+      </c>
+      <c r="H35" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="J35" s="2">
+        <v>4</v>
+      </c>
       <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-    </row>
-    <row r="36" spans="1:12">
-      <c r="A36" s="2"/>
+      <c r="L35" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="27">
+      <c r="A36" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="B36" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A36,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
+        <v>Rows</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="G36" s="2">
+        <v>4</v>
+      </c>
+      <c r="H36" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="J36" s="2">
+        <v>5</v>
+      </c>
       <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-    </row>
-    <row r="37" spans="1:12">
-      <c r="A37" s="2"/>
+      <c r="L36" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="27">
+      <c r="A37" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="B37" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A37,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
+        <v>Formula Bot</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G37" s="2">
+        <v>4</v>
+      </c>
+      <c r="H37" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="J37" s="2">
+        <v>4</v>
+      </c>
       <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-    </row>
-    <row r="38" spans="1:12">
-      <c r="A38" s="2"/>
+      <c r="L37" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="27">
+      <c r="A38" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="B38" s="2" t="str">
         <f>IFERROR(INDEX('01_Компании'!$B$4:$B$103,MATCH(A38,'01_Компании'!$A$4:$A$103,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
+        <v>Microsoft 365 Copilot</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="G38" s="2">
+        <v>5</v>
+      </c>
+      <c r="H38" s="5">
+        <v>46298</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="J38" s="2">
+        <v>5</v>
+      </c>
       <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
+      <c r="L38" s="2" t="s">
+        <v>475</v>
+      </c>
     </row>
     <row r="39" spans="1:12">
       <c r="A39" s="2"/>

</xml_diff>